<commit_message>
Resultados v1.2: re-run completo del pipeline (01-18 + checklist STROBE)
Base analitica 25 088 adultos (B7: -1 excluido, 20 conservan su PA real y dejan de contar como
hipertensos; denominador HTA-ESH 7 756 -> 7 735). Cobertura nacional 2 466-2 469 municipios
(99,5-99,6%; A2 recupera los 18 de CLUES). Cifras nacionales directas se mueven <= 0,2 pp:
prevalencia ESH 27,3 (26,2-28,4), conciencia 65,9, tratamiento 81,0, control 64,0 / 40,6.
Reclasificacion: mediana -23,2 / -25,3 pp, DE 1,6. OR de pobreza por +10 pp: 0,92-0,94, los 4 IC
excluyen el 1. Phi: 0,12 / 0,06 / 0,81 / 0,65 / 0,51. Los n de los modelos: 7 727 / 11 583 /
5 203 / 4 382 (C1). Figuras 1-3, S1-S2, tablas y checklist regenerados desde estos outputs.

El manuscrito (.md) sigue con cifras v1.1: la Fase C se hace con
_TRABAJO_INTERNO/diff_v11_v12.md delante (no versionado).
</commit_message>
<xml_diff>
--- a/FIGURAS/DATOS/Fig1_datos.xlsx
+++ b/FIGURAS/DATOS/Fig1_datos.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -377,55 +377,60 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>excl_lectura_fuera_de_rango</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>excl_lectura_invertida</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>excl_sin_bp_valida</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>excl_embarazo_actual</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>excl_sin_peso</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>n_final</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>n_hta_esh</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>n_hta_aha</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>n_diagnosticados</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>n_tratados</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>integrantes_match_pct</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>escolaridad_no_na_pct</t>
         </is>
@@ -442,39 +447,42 @@
         <v>13402</v>
       </c>
       <c r="D2">
-        <v>8195</v>
+        <v>8194</v>
       </c>
       <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
         <v>0</v>
       </c>
-      <c r="F2">
-        <v>5207</v>
-      </c>
       <c r="G2">
+        <v>5208</v>
+      </c>
+      <c r="H2">
         <v>127</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>1</v>
       </c>
-      <c r="I2">
-        <v>8067</v>
-      </c>
       <c r="J2">
-        <v>2368</v>
+        <v>8066</v>
       </c>
       <c r="K2">
-        <v>3630</v>
+        <v>2364</v>
       </c>
       <c r="L2">
-        <v>1608</v>
+        <v>3626</v>
       </c>
       <c r="M2">
-        <v>1349</v>
+        <v>1607</v>
       </c>
       <c r="N2">
-        <v>100</v>
+        <v>1348</v>
       </c>
       <c r="O2">
+        <v>100</v>
+      </c>
+      <c r="P2">
         <v>100</v>
       </c>
     </row>
@@ -489,39 +497,42 @@
         <v>11913</v>
       </c>
       <c r="D3">
-        <v>8750</v>
+        <v>8746</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
         <v>3167</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>107</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>0</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>8639</v>
       </c>
-      <c r="J3">
-        <v>2789</v>
-      </c>
       <c r="K3">
-        <v>4183</v>
+        <v>2786</v>
       </c>
       <c r="L3">
+        <v>4181</v>
+      </c>
+      <c r="M3">
         <v>1778</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>1529</v>
       </c>
-      <c r="N3">
-        <v>100</v>
-      </c>
       <c r="O3">
+        <v>100</v>
+      </c>
+      <c r="P3">
         <v>100</v>
       </c>
     </row>
@@ -536,39 +547,42 @@
         <v>6772</v>
       </c>
       <c r="D4">
-        <v>3147</v>
+        <v>3144</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
         <v>3628</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>36</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>0</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>3108</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>1017</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>1505</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <v>692</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>568</v>
       </c>
-      <c r="N4">
-        <v>100</v>
-      </c>
       <c r="O4">
+        <v>100</v>
+      </c>
+      <c r="P4">
         <v>100</v>
       </c>
     </row>
@@ -583,39 +597,42 @@
         <v>12924</v>
       </c>
       <c r="D5">
-        <v>5347</v>
+        <v>5326</v>
       </c>
       <c r="E5">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
         <v>7598</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>51</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>0</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>5275</v>
       </c>
-      <c r="J5">
-        <v>1582</v>
-      </c>
       <c r="K5">
-        <v>2293</v>
+        <v>1568</v>
       </c>
       <c r="L5">
+        <v>2285</v>
+      </c>
+      <c r="M5">
         <v>1126</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>943</v>
       </c>
-      <c r="N5">
-        <v>100</v>
-      </c>
       <c r="O5">
+        <v>100</v>
+      </c>
+      <c r="P5">
         <v>100</v>
       </c>
     </row>

</xml_diff>